<commit_message>
Update Aura forecast exports and add new analytics visualizations
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/artifacts/aura-forecast/public/exports/DAILY_FORECAST_2026-09-01.xlsx
+++ b/artifacts/aura-forecast/public/exports/DAILY_FORECAST_2026-09-01.xlsx
@@ -3,6 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="Daily_Forecast" sheetId="1" r:id="rId1"/>
+    <sheet name="Analysis_Stats" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -72,27 +73,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>24.881431</t>
+          <t>24.707413</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>73.080246</t>
+          <t>70.771741</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>970.042216</t>
+          <t>970.099624</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>23.588545</t>
+          <t>23.495936</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>331.1586</t>
+          <t>329.2403</t>
         </is>
       </c>
     </row>
@@ -104,27 +105,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>24.710004</t>
+          <t>24.449293</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>73.20397</t>
+          <t>71.991273</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>969.444974</t>
+          <t>969.343185</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>23.414437</t>
+          <t>23.259301</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>330.7183</t>
+          <t>329.9432</t>
         </is>
       </c>
     </row>
@@ -136,27 +137,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>24.482862</t>
+          <t>24.210417</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>73.712959</t>
+          <t>73.502626</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>969.059331</t>
+          <t>968.949463</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>23.206653</t>
+          <t>22.940393</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>330.8268</t>
+          <t>330.0819</t>
         </is>
       </c>
     </row>
@@ -168,27 +169,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>24.582908</t>
+          <t>24.401874</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>74.238497</t>
+          <t>74.874234</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>969.180407</t>
+          <t>969.158344</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>23.204286</t>
+          <t>23.171106</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>330.5573</t>
+          <t>332.3108</t>
         </is>
       </c>
     </row>
@@ -200,27 +201,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>24.470863</t>
+          <t>24.237009</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>74.89093</t>
+          <t>74.267074</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>969.445453</t>
+          <t>969.510289</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>23.085693</t>
+          <t>23.164964</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>330.9641</t>
+          <t>332.9734</t>
         </is>
       </c>
     </row>
@@ -232,27 +233,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>24.366099</t>
+          <t>24.029233</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>75.841067</t>
+          <t>74.118768</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>969.96548</t>
+          <t>970.075745</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>22.920364</t>
+          <t>22.74643</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>331.2278</t>
+          <t>330.4197</t>
         </is>
       </c>
     </row>
@@ -264,27 +265,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>24.51034</t>
+          <t>24.154912</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>75.788316</t>
+          <t>73.831917</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>970.573631</t>
+          <t>970.526118</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>23.041569</t>
+          <t>22.747001</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>331.3325</t>
+          <t>329.173</t>
         </is>
       </c>
     </row>
@@ -296,27 +297,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>24.911694</t>
+          <t>24.647275</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>73.962036</t>
+          <t>69.520525</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>971.226553</t>
+          <t>971.114795</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>23.531957</t>
+          <t>23.33741</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>331.2249</t>
+          <t>326.7314</t>
         </is>
       </c>
     </row>
@@ -328,27 +329,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>25.641859</t>
+          <t>25.595685</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>70.784953</t>
+          <t>69.1575</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>971.628974</t>
+          <t>971.792772</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>24.439237</t>
+          <t>24.296746</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>331.1475</t>
+          <t>328.4732</t>
         </is>
       </c>
     </row>
@@ -360,27 +361,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>26.333294</t>
+          <t>26.277507</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>66.591797</t>
+          <t>64.764636</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>971.698276</t>
+          <t>971.718622</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>25.076853</t>
+          <t>25.030172</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>327.5307</t>
+          <t>325.6191</t>
         </is>
       </c>
     </row>
@@ -392,27 +393,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>27.107713</t>
+          <t>27.080325</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>61.722927</t>
+          <t>57.002109</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>971.250674</t>
+          <t>970.977891</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>26.093355</t>
+          <t>26.161077</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>326.129</t>
+          <t>322.009</t>
         </is>
       </c>
     </row>
@@ -424,27 +425,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>27.885193</t>
+          <t>28.09888</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>58.171655</t>
+          <t>53.322216</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>970.577295</t>
+          <t>970.275669</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>26.788487</t>
+          <t>26.819623</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>322.8284</t>
+          <t>316.2968</t>
         </is>
       </c>
     </row>
@@ -456,27 +457,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28.535922</t>
+          <t>28.925149</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>54.65175</t>
+          <t>47.121092</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>969.566332</t>
+          <t>969.150772</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>27.170978</t>
+          <t>27.156796</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>317.3688</t>
+          <t>306.1734</t>
         </is>
       </c>
     </row>
@@ -488,27 +489,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>29.194265</t>
+          <t>30.303378</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>52.151046</t>
+          <t>41.707615</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>968.683527</t>
+          <t>968.273112</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>28.125784</t>
+          <t>28.242852</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>318.6614</t>
+          <t>300.0552</t>
         </is>
       </c>
     </row>
@@ -520,27 +521,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>29.377491</t>
+          <t>30.817592</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>53.230873</t>
+          <t>45.74339</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>968.246109</t>
+          <t>968.136528</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>28.36664</t>
+          <t>28.720987</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>320.5639</t>
+          <t>304.8776</t>
         </is>
       </c>
     </row>
@@ -552,27 +553,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28.98218</t>
+          <t>29.422877</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>52.435851</t>
+          <t>46.580774</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>967.784203</t>
+          <t>967.719689</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>28.041109</t>
+          <t>27.880798</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>319.5089</t>
+          <t>308.3337</t>
         </is>
       </c>
     </row>
@@ -584,27 +585,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28.199278</t>
+          <t>28.773703</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>53.082569</t>
+          <t>49.766859</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>967.718595</t>
+          <t>967.641062</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>27.389637</t>
+          <t>27.207817</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>319.9711</t>
+          <t>310.1588</t>
         </is>
       </c>
     </row>
@@ -616,27 +617,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>27.34475</t>
+          <t>27.906887</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>57.724685</t>
+          <t>55.714137</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>968.246527</t>
+          <t>968.3945</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>26.590898</t>
+          <t>26.526403</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>323.9457</t>
+          <t>316.834</t>
         </is>
       </c>
     </row>
@@ -648,27 +649,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>26.674012</t>
+          <t>27.196635</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>64.07608</t>
+          <t>62.921389</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>969.069649</t>
+          <t>969.11654</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>25.91429</t>
+          <t>25.911451</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>329.5872</t>
+          <t>324.2487</t>
         </is>
       </c>
     </row>
@@ -680,27 +681,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>26.196524</t>
+          <t>26.624783</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>67.423792</t>
+          <t>69.327201</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>969.807284</t>
+          <t>970.09423</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>25.282803</t>
+          <t>25.083106</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>331.0089</t>
+          <t>327.7341</t>
         </is>
       </c>
     </row>
@@ -712,27 +713,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>25.890578</t>
+          <t>26.283601</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>70.660564</t>
+          <t>71.998102</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>970.515662</t>
+          <t>970.778455</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>24.869598</t>
+          <t>24.819582</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>333.1135</t>
+          <t>331.0025</t>
         </is>
       </c>
     </row>
@@ -744,27 +745,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25.551221</t>
+          <t>25.604899</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>71.566683</t>
+          <t>69.84602</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>970.929014</t>
+          <t>970.925783</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>24.394734</t>
+          <t>23.938245</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>332.3306</t>
+          <t>325.5971</t>
         </is>
       </c>
     </row>
@@ -776,27 +777,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25.227838</t>
+          <t>25.184776</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>72.143637</t>
+          <t>70.63538</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>971.033641</t>
+          <t>970.849908</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>23.98776</t>
+          <t>23.453257</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>331.6173</t>
+          <t>325.0272</t>
         </is>
       </c>
     </row>
@@ -808,27 +809,214 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>24.972018</t>
+          <t>25.049697</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>72.601228</t>
+          <t>72.205043</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>970.545686</t>
+          <t>970.383701</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>23.700834</t>
+          <t>23.076122</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>331.1838</t>
+          <t>323.9097</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Analysis item</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Forecast rows in package</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Forecast profile</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>weekday × hour training profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Forecast target</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>refractivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Visual asset</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>analytics/data_quality_missingness.svg</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Missing percentage by variable</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>analytics/data_quality_outliers.svg</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Flagged outlier counts by variable</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>analytics/hist_temperature.svg</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Temperature histogram</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>analytics/hist_pressure.svg</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pressure histogram</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>analytics/hist_refractivity.svg</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Refractivity histogram</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>analytics/correlation_refractivity.svg</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Predictor correlation with refractivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>analytics/daily_refractivity.svg</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Daily refractivity trend</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>analytics/monthly_forecast.svg</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Monthly forecast comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>analytics/validation_metrics.svg</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Chronological validation scorecard</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>analytics/training_holdout_rows.svg</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Training, holdout, and validation counts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix heatIndex train/validation mismatch - R2 -4.70 to 0.91
</commit_message>
<xml_diff>
--- a/artifacts/aura-forecast/public/exports/DAILY_FORECAST_2026-09-01.xlsx
+++ b/artifacts/aura-forecast/public/exports/DAILY_FORECAST_2026-09-01.xlsx
@@ -93,7 +93,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>329.2403</t>
+          <t>346.0705</t>
         </is>
       </c>
     </row>
@@ -125,7 +125,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>329.9432</t>
+          <t>346.6209</t>
         </is>
       </c>
     </row>
@@ -157,7 +157,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>330.0819</t>
+          <t>348.1796</t>
         </is>
       </c>
     </row>
@@ -189,7 +189,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>332.3108</t>
+          <t>350.5689</t>
         </is>
       </c>
     </row>
@@ -221,7 +221,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>332.9734</t>
+          <t>349.3775</t>
         </is>
       </c>
     </row>
@@ -253,7 +253,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>330.4197</t>
+          <t>349.785</t>
         </is>
       </c>
     </row>
@@ -285,7 +285,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>329.173</t>
+          <t>350.6281</t>
         </is>
       </c>
     </row>
@@ -317,7 +317,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>326.7314</t>
+          <t>345.9192</t>
         </is>
       </c>
     </row>
@@ -349,7 +349,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>328.4732</t>
+          <t>348.3018</t>
         </is>
       </c>
     </row>
@@ -381,7 +381,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>325.6191</t>
+          <t>343.8497</t>
         </is>
       </c>
     </row>
@@ -413,7 +413,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>322.009</t>
+          <t>333.8168</t>
         </is>
       </c>
     </row>
@@ -445,7 +445,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>316.2968</t>
+          <t>331.5338</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>306.1734</t>
+          <t>325.0595</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>300.0552</t>
+          <t>320.3419</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>304.8776</t>
+          <t>327.6807</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>308.3337</t>
+          <t>325.1251</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>310.1588</t>
+          <t>328.4632</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>316.834</t>
+          <t>335.1708</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>324.2487</t>
+          <t>344.025</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>327.7341</t>
+          <t>352.5238</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>331.0025</t>
+          <t>355.0386</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>325.5971</t>
+          <t>349.9819</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>325.0272</t>
+          <t>349.5296</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>323.9097</t>
+          <t>351.0883</t>
         </is>
       </c>
     </row>

</xml_diff>